<commit_message>
fix(excel): refined layout with specific font sizes and dynamic sign-off boxes
</commit_message>
<xml_diff>
--- a/docs/samples/written/【Fハウス】訪問施術サービス申込書.xlsx
+++ b/docs/samples/written/【Fハウス】訪問施術サービス申込書.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hannanplage.sharepoint.com/sites/msteams_407f57-94/Shared Documents/訪問施術/Ｆハウス/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/cd35f0bba0eb985b/デスクトップ/VEXUM/プラージュ様/-OCR-main/-OCR-main/docs/samples/written/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{9AC4E2FC-E607-4C7F-B889-09B397EE049A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{19F3334E-992E-409D-AB4F-249C81AFF9DC}"/>
+  <xr:revisionPtr revIDLastSave="10" documentId="13_ncr:1_{9AC4E2FC-E607-4C7F-B889-09B397EE049A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C7D5B176-3220-47FE-AE84-D673B7C86505}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{8545FFEA-CFB0-4F4D-92CA-7457519C6A3D}"/>
   </bookViews>
@@ -42,9 +42,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="49">
   <si>
-    <t>【訪問理美容サービス　申込書】</t>
-  </si>
-  <si>
     <t>確認
 サイン欄</t>
     <rPh sb="0" eb="2">
@@ -318,6 +315,10 @@
   </si>
   <si>
     <t>　Fハウス</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>【訪問理美容サービス　申込書】</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -1533,23 +1534,11 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="5" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="6" fontId="21" fillId="4" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="48" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1559,16 +1548,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="5" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1628,10 +1607,10 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="6" fontId="21" fillId="4" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1639,6 +1618,28 @@
     </xf>
     <xf numFmtId="0" fontId="22" fillId="3" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1861,25 +1862,25 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:V59"/>
-  <sheetFormatPr defaultColWidth="12.5546875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="3.88671875" style="6" customWidth="1"/>
-    <col min="2" max="2" width="8.6640625" style="6" customWidth="1"/>
-    <col min="3" max="5" width="12.5546875" style="6" customWidth="1"/>
-    <col min="6" max="12" width="11.44140625" style="6" customWidth="1"/>
-    <col min="13" max="13" width="12.5546875" style="6"/>
-    <col min="14" max="16" width="10.109375" style="6" customWidth="1"/>
-    <col min="17" max="19" width="15.77734375" style="6" customWidth="1"/>
-    <col min="20" max="20" width="15.88671875" style="6" customWidth="1"/>
-    <col min="21" max="21" width="16.6640625" style="6" customWidth="1"/>
-    <col min="22" max="22" width="43.5546875" style="6" customWidth="1"/>
-    <col min="23" max="16384" width="12.5546875" style="6"/>
+    <col min="1" max="1" width="3.90625" style="6" customWidth="1"/>
+    <col min="2" max="2" width="8.6328125" style="6" customWidth="1"/>
+    <col min="3" max="5" width="12.54296875" style="6" customWidth="1"/>
+    <col min="6" max="12" width="11.453125" style="6" customWidth="1"/>
+    <col min="13" max="13" width="12.54296875" style="6"/>
+    <col min="14" max="16" width="10.08984375" style="6" customWidth="1"/>
+    <col min="17" max="19" width="15.81640625" style="6" customWidth="1"/>
+    <col min="20" max="20" width="15.90625" style="6" customWidth="1"/>
+    <col min="21" max="21" width="16.6328125" style="6" customWidth="1"/>
+    <col min="22" max="22" width="43.54296875" style="6" customWidth="1"/>
+    <col min="23" max="16384" width="12.54296875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" ht="30.6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:22" ht="31.5" x14ac:dyDescent="0.45">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="C1" s="3"/>
       <c r="D1" s="1"/>
@@ -1898,13 +1899,13 @@
       <c r="Q1" s="5"/>
       <c r="R1" s="4"/>
       <c r="S1" s="4"/>
-      <c r="T1" s="91" t="s">
-        <v>1</v>
-      </c>
-      <c r="U1" s="92"/>
+      <c r="T1" s="83" t="s">
+        <v>0</v>
+      </c>
+      <c r="U1" s="84"/>
       <c r="V1" s="1"/>
     </row>
-    <row r="2" spans="1:22" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:22" ht="13.5" x14ac:dyDescent="0.3">
       <c r="A2" s="7"/>
       <c r="D2" s="7"/>
       <c r="E2" s="7"/>
@@ -1922,50 +1923,50 @@
       <c r="Q2" s="7"/>
       <c r="R2" s="7"/>
       <c r="S2" s="7"/>
-      <c r="T2" s="93"/>
-      <c r="U2" s="94"/>
+      <c r="T2" s="85"/>
+      <c r="U2" s="86"/>
       <c r="V2" s="7"/>
     </row>
-    <row r="3" spans="1:22" ht="19.2" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:22" ht="20" thickBot="1" x14ac:dyDescent="0.5">
       <c r="A3" s="8"/>
       <c r="B3" s="8" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C3" s="8"/>
       <c r="D3" s="8"/>
       <c r="E3" s="8"/>
       <c r="F3" s="8"/>
       <c r="H3" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="I3" s="10" t="s">
         <v>47</v>
-      </c>
-      <c r="I3" s="10" t="s">
-        <v>48</v>
       </c>
       <c r="J3" s="9"/>
       <c r="K3" s="9"/>
       <c r="L3" s="9"/>
       <c r="M3" s="9"/>
       <c r="O3" s="9" t="s">
+        <v>2</v>
+      </c>
+      <c r="P3" s="10" t="s">
         <v>3</v>
-      </c>
-      <c r="P3" s="10" t="s">
-        <v>4</v>
       </c>
       <c r="Q3" s="10"/>
       <c r="R3" s="9"/>
       <c r="S3" s="9"/>
       <c r="T3" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="U3" s="12" t="s">
         <v>5</v>
-      </c>
-      <c r="U3" s="12" t="s">
-        <v>6</v>
       </c>
       <c r="V3" s="8"/>
     </row>
     <row r="4" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A4" s="7"/>
       <c r="B4" s="8" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C4" s="8"/>
       <c r="D4" s="8"/>
@@ -1984,17 +1985,17 @@
       <c r="R4" s="7"/>
       <c r="S4" s="7"/>
       <c r="T4" s="13" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="U4" s="14" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V4" s="7"/>
     </row>
     <row r="5" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A5" s="7"/>
       <c r="B5" s="8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
@@ -2013,7 +2014,7 @@
     <row r="6" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A6" s="7"/>
       <c r="B6" s="8" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C6" s="8"/>
       <c r="D6" s="8"/>
@@ -2038,7 +2039,7 @@
     <row r="7" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A7" s="7"/>
       <c r="B7" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C7" s="8"/>
       <c r="D7" s="8"/>
@@ -2063,7 +2064,7 @@
     <row r="8" spans="1:22" ht="18" x14ac:dyDescent="0.3">
       <c r="A8" s="7"/>
       <c r="B8" s="8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C8" s="8"/>
       <c r="D8" s="8"/>
@@ -2085,14 +2086,14 @@
       <c r="U8" s="71"/>
       <c r="V8" s="7"/>
     </row>
-    <row r="9" spans="1:22" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:22" ht="18.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="7"/>
-      <c r="B9" s="117" t="s">
+      <c r="B9" s="109" t="s">
+        <v>43</v>
+      </c>
+      <c r="C9" s="109"/>
+      <c r="D9" s="72" t="s">
         <v>44</v>
-      </c>
-      <c r="C9" s="117"/>
-      <c r="D9" s="72" t="s">
-        <v>45</v>
       </c>
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
@@ -2123,7 +2124,7 @@
       <c r="U10" s="73"/>
       <c r="V10" s="7"/>
     </row>
-    <row r="11" spans="1:22" ht="16.2" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:22" ht="16" x14ac:dyDescent="0.3">
       <c r="A11" s="7"/>
       <c r="F11" s="7"/>
       <c r="G11" s="7"/>
@@ -2145,96 +2146,96 @@
     </row>
     <row r="12" spans="1:22" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="15"/>
-      <c r="B12" s="95" t="s">
+      <c r="B12" s="87" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" s="89" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="97" t="s">
+      <c r="D12" s="91" t="s">
         <v>11</v>
       </c>
-      <c r="D12" s="99" t="s">
+      <c r="E12" s="92"/>
+      <c r="F12" s="95" t="s">
         <v>12</v>
       </c>
-      <c r="E12" s="100"/>
-      <c r="F12" s="103" t="s">
+      <c r="G12" s="96"/>
+      <c r="H12" s="96"/>
+      <c r="I12" s="96"/>
+      <c r="J12" s="96"/>
+      <c r="K12" s="96"/>
+      <c r="L12" s="97"/>
+      <c r="M12" s="98" t="s">
         <v>13</v>
       </c>
-      <c r="G12" s="104"/>
-      <c r="H12" s="104"/>
-      <c r="I12" s="104"/>
-      <c r="J12" s="104"/>
-      <c r="K12" s="104"/>
-      <c r="L12" s="105"/>
-      <c r="M12" s="106" t="s">
+      <c r="N12" s="87" t="s">
         <v>14</v>
       </c>
-      <c r="N12" s="95" t="s">
+      <c r="O12" s="100"/>
+      <c r="P12" s="100"/>
+      <c r="Q12" s="101" t="s">
+        <v>45</v>
+      </c>
+      <c r="R12" s="101" t="s">
         <v>15</v>
       </c>
-      <c r="O12" s="108"/>
-      <c r="P12" s="108"/>
-      <c r="Q12" s="109" t="s">
-        <v>46</v>
-      </c>
-      <c r="R12" s="109" t="s">
+      <c r="S12" s="101" t="s">
         <v>16</v>
       </c>
-      <c r="S12" s="109" t="s">
+      <c r="T12" s="102" t="s">
         <v>17</v>
       </c>
-      <c r="T12" s="110" t="s">
+      <c r="U12" s="106" t="s">
         <v>18</v>
       </c>
-      <c r="U12" s="114" t="s">
+      <c r="V12" s="107"/>
+    </row>
+    <row r="13" spans="1:22" ht="30" x14ac:dyDescent="0.35">
+      <c r="A13" s="15"/>
+      <c r="B13" s="88"/>
+      <c r="C13" s="90"/>
+      <c r="D13" s="93"/>
+      <c r="E13" s="94"/>
+      <c r="F13" s="16" t="s">
         <v>19</v>
       </c>
-      <c r="V12" s="115"/>
-    </row>
-    <row r="13" spans="1:22" ht="30" x14ac:dyDescent="0.3">
-      <c r="A13" s="15"/>
-      <c r="B13" s="96"/>
-      <c r="C13" s="98"/>
-      <c r="D13" s="101"/>
-      <c r="E13" s="102"/>
-      <c r="F13" s="16" t="s">
+      <c r="G13" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="G13" s="17" t="s">
+      <c r="H13" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="H13" s="18" t="s">
+      <c r="I13" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="I13" s="17" t="s">
+      <c r="J13" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="J13" s="18" t="s">
+      <c r="K13" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="K13" s="18" t="s">
+      <c r="L13" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="M13" s="99"/>
+      <c r="N13" s="103" t="s">
         <v>25</v>
       </c>
-      <c r="L13" s="18" t="s">
-        <v>40</v>
-      </c>
-      <c r="M13" s="107"/>
-      <c r="N13" s="111" t="s">
-        <v>26</v>
-      </c>
-      <c r="O13" s="112"/>
-      <c r="P13" s="113"/>
-      <c r="Q13" s="98"/>
-      <c r="R13" s="98"/>
-      <c r="S13" s="98"/>
-      <c r="T13" s="96"/>
-      <c r="U13" s="115"/>
-      <c r="V13" s="115"/>
-    </row>
-    <row r="14" spans="1:22" ht="16.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="O13" s="104"/>
+      <c r="P13" s="105"/>
+      <c r="Q13" s="90"/>
+      <c r="R13" s="90"/>
+      <c r="S13" s="90"/>
+      <c r="T13" s="88"/>
+      <c r="U13" s="107"/>
+      <c r="V13" s="107"/>
+    </row>
+    <row r="14" spans="1:22" ht="16.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A14" s="15"/>
-      <c r="B14" s="96"/>
-      <c r="C14" s="98"/>
-      <c r="D14" s="101"/>
-      <c r="E14" s="102"/>
+      <c r="B14" s="88"/>
+      <c r="C14" s="90"/>
+      <c r="D14" s="93"/>
+      <c r="E14" s="94"/>
       <c r="F14" s="19">
         <v>2000</v>
       </c>
@@ -2256,63 +2257,63 @@
       <c r="L14" s="20">
         <v>0</v>
       </c>
-      <c r="M14" s="107"/>
+      <c r="M14" s="99"/>
       <c r="N14" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="O14" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="O14" s="22" t="s">
+      <c r="P14" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="P14" s="23" t="s">
+      <c r="Q14" s="90"/>
+      <c r="R14" s="90"/>
+      <c r="S14" s="90"/>
+      <c r="T14" s="88"/>
+      <c r="U14" s="108"/>
+      <c r="V14" s="108"/>
+    </row>
+    <row r="15" spans="1:22" s="29" customFormat="1" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="15"/>
+      <c r="B15" s="110" t="s">
         <v>29</v>
       </c>
-      <c r="Q14" s="98"/>
-      <c r="R14" s="98"/>
-      <c r="S14" s="98"/>
-      <c r="T14" s="96"/>
-      <c r="U14" s="116"/>
-      <c r="V14" s="116"/>
-    </row>
-    <row r="15" spans="1:22" s="29" customFormat="1" ht="16.8" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="15"/>
-      <c r="B15" s="87" t="s">
-        <v>30</v>
-      </c>
-      <c r="C15" s="88"/>
-      <c r="D15" s="120">
+      <c r="C15" s="111"/>
+      <c r="D15" s="112">
         <f>COUNTA(D17:E59)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="121"/>
-      <c r="F15" s="118">
+      <c r="E15" s="113"/>
+      <c r="F15" s="77">
         <f t="shared" ref="F15:L15" si="0">COUNTIF(F17:F59,"〇")</f>
         <v>0</v>
       </c>
-      <c r="G15" s="118">
+      <c r="G15" s="77">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H15" s="118">
+      <c r="H15" s="77">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="I15" s="118">
+      <c r="I15" s="77">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="J15" s="118">
+      <c r="J15" s="77">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K15" s="118">
+      <c r="K15" s="77">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L15" s="118">
+      <c r="L15" s="77">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="M15" s="119">
+      <c r="M15" s="78">
         <f>SUM(M17:M59)</f>
         <v>0</v>
       </c>
@@ -2323,65 +2324,65 @@
       <c r="R15" s="27"/>
       <c r="S15" s="28"/>
       <c r="T15" s="28"/>
-      <c r="U15" s="81"/>
-      <c r="V15" s="82"/>
-    </row>
-    <row r="16" spans="1:22" ht="16.2" x14ac:dyDescent="0.3">
+      <c r="U15" s="118"/>
+      <c r="V15" s="119"/>
+    </row>
+    <row r="16" spans="1:22" ht="16" x14ac:dyDescent="0.35">
       <c r="A16" s="30"/>
       <c r="B16" s="57" t="s">
+        <v>30</v>
+      </c>
+      <c r="C16" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="31" t="s">
+      <c r="D16" s="114" t="s">
         <v>32</v>
       </c>
-      <c r="D16" s="89" t="s">
+      <c r="E16" s="115"/>
+      <c r="F16" s="32" t="s">
         <v>33</v>
-      </c>
-      <c r="E16" s="90"/>
-      <c r="F16" s="32" t="s">
-        <v>34</v>
       </c>
       <c r="G16" s="33"/>
       <c r="H16" s="33"/>
       <c r="I16" s="33"/>
       <c r="J16" s="33" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="K16" s="33"/>
       <c r="L16" s="33" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M16" s="34">
         <v>4500</v>
       </c>
       <c r="N16" s="35" t="s">
+        <v>34</v>
+      </c>
+      <c r="O16" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="O16" s="36" t="s">
+      <c r="P16" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="P16" s="37" t="s">
-        <v>37</v>
-      </c>
       <c r="Q16" s="38" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="R16" s="38" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="S16" s="39"/>
       <c r="T16" s="39"/>
-      <c r="U16" s="79"/>
-      <c r="V16" s="80"/>
-    </row>
-    <row r="17" spans="1:22" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="U16" s="120"/>
+      <c r="V16" s="121"/>
+    </row>
+    <row r="17" spans="1:22" ht="37.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="7"/>
       <c r="B17" s="58">
         <v>1</v>
       </c>
       <c r="C17" s="56"/>
-      <c r="D17" s="83"/>
-      <c r="E17" s="84"/>
+      <c r="D17" s="79"/>
+      <c r="E17" s="80"/>
       <c r="F17" s="61"/>
       <c r="G17" s="62"/>
       <c r="H17" s="62"/>
@@ -2399,22 +2400,22 @@
       <c r="Q17" s="44"/>
       <c r="R17" s="44"/>
       <c r="S17" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T17" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U17" s="78"/>
-      <c r="V17" s="78"/>
-    </row>
-    <row r="18" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U17" s="116"/>
+      <c r="V17" s="116"/>
+    </row>
+    <row r="18" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="7"/>
       <c r="B18" s="59">
         <v>2</v>
       </c>
       <c r="C18" s="55"/>
-      <c r="D18" s="85"/>
-      <c r="E18" s="86"/>
+      <c r="D18" s="81"/>
+      <c r="E18" s="82"/>
       <c r="F18" s="63"/>
       <c r="G18" s="64"/>
       <c r="H18" s="64"/>
@@ -2432,22 +2433,22 @@
       <c r="Q18" s="52"/>
       <c r="R18" s="52"/>
       <c r="S18" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T18" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U18" s="77"/>
-      <c r="V18" s="77"/>
-    </row>
-    <row r="19" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U18" s="117"/>
+      <c r="V18" s="117"/>
+    </row>
+    <row r="19" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="7"/>
       <c r="B19" s="58">
         <v>3</v>
       </c>
       <c r="C19" s="56"/>
-      <c r="D19" s="83"/>
-      <c r="E19" s="84"/>
+      <c r="D19" s="79"/>
+      <c r="E19" s="80"/>
       <c r="F19" s="61"/>
       <c r="G19" s="62"/>
       <c r="H19" s="62"/>
@@ -2465,22 +2466,22 @@
       <c r="Q19" s="47"/>
       <c r="R19" s="47"/>
       <c r="S19" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T19" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U19" s="78"/>
-      <c r="V19" s="78"/>
-    </row>
-    <row r="20" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U19" s="116"/>
+      <c r="V19" s="116"/>
+    </row>
+    <row r="20" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="7"/>
       <c r="B20" s="59">
         <v>4</v>
       </c>
       <c r="C20" s="55"/>
-      <c r="D20" s="85"/>
-      <c r="E20" s="86"/>
+      <c r="D20" s="81"/>
+      <c r="E20" s="82"/>
       <c r="F20" s="63"/>
       <c r="G20" s="64"/>
       <c r="H20" s="64"/>
@@ -2498,22 +2499,22 @@
       <c r="Q20" s="75"/>
       <c r="R20" s="48"/>
       <c r="S20" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T20" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U20" s="77"/>
-      <c r="V20" s="77"/>
-    </row>
-    <row r="21" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U20" s="117"/>
+      <c r="V20" s="117"/>
+    </row>
+    <row r="21" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="7"/>
       <c r="B21" s="58">
         <v>5</v>
       </c>
       <c r="C21" s="56"/>
-      <c r="D21" s="83"/>
-      <c r="E21" s="84"/>
+      <c r="D21" s="79"/>
+      <c r="E21" s="80"/>
       <c r="F21" s="61"/>
       <c r="G21" s="62"/>
       <c r="H21" s="62"/>
@@ -2531,22 +2532,22 @@
       <c r="Q21" s="76"/>
       <c r="R21" s="40"/>
       <c r="S21" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T21" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U21" s="78"/>
-      <c r="V21" s="78"/>
-    </row>
-    <row r="22" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U21" s="116"/>
+      <c r="V21" s="116"/>
+    </row>
+    <row r="22" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="7"/>
       <c r="B22" s="59">
         <v>6</v>
       </c>
       <c r="C22" s="55"/>
-      <c r="D22" s="85"/>
-      <c r="E22" s="86"/>
+      <c r="D22" s="81"/>
+      <c r="E22" s="82"/>
       <c r="F22" s="63"/>
       <c r="G22" s="64"/>
       <c r="H22" s="64"/>
@@ -2564,22 +2565,22 @@
       <c r="Q22" s="75"/>
       <c r="R22" s="48"/>
       <c r="S22" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T22" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U22" s="77"/>
-      <c r="V22" s="77"/>
-    </row>
-    <row r="23" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U22" s="117"/>
+      <c r="V22" s="117"/>
+    </row>
+    <row r="23" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="7"/>
       <c r="B23" s="58">
         <v>7</v>
       </c>
       <c r="C23" s="56"/>
-      <c r="D23" s="83"/>
-      <c r="E23" s="84"/>
+      <c r="D23" s="79"/>
+      <c r="E23" s="80"/>
       <c r="F23" s="61"/>
       <c r="G23" s="62"/>
       <c r="H23" s="62"/>
@@ -2597,22 +2598,22 @@
       <c r="Q23" s="76"/>
       <c r="R23" s="40"/>
       <c r="S23" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T23" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U23" s="78"/>
-      <c r="V23" s="78"/>
-    </row>
-    <row r="24" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U23" s="116"/>
+      <c r="V23" s="116"/>
+    </row>
+    <row r="24" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="7"/>
       <c r="B24" s="59">
         <v>8</v>
       </c>
       <c r="C24" s="55"/>
-      <c r="D24" s="85"/>
-      <c r="E24" s="86"/>
+      <c r="D24" s="81"/>
+      <c r="E24" s="82"/>
       <c r="F24" s="63"/>
       <c r="G24" s="64"/>
       <c r="H24" s="64"/>
@@ -2630,22 +2631,22 @@
       <c r="Q24" s="75"/>
       <c r="R24" s="48"/>
       <c r="S24" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T24" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U24" s="77"/>
-      <c r="V24" s="77"/>
-    </row>
-    <row r="25" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U24" s="117"/>
+      <c r="V24" s="117"/>
+    </row>
+    <row r="25" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="7"/>
       <c r="B25" s="58">
         <v>9</v>
       </c>
       <c r="C25" s="56"/>
-      <c r="D25" s="83"/>
-      <c r="E25" s="84"/>
+      <c r="D25" s="79"/>
+      <c r="E25" s="80"/>
       <c r="F25" s="61"/>
       <c r="G25" s="62"/>
       <c r="H25" s="62"/>
@@ -2663,22 +2664,22 @@
       <c r="Q25" s="76"/>
       <c r="R25" s="40"/>
       <c r="S25" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T25" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U25" s="78"/>
-      <c r="V25" s="78"/>
-    </row>
-    <row r="26" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U25" s="116"/>
+      <c r="V25" s="116"/>
+    </row>
+    <row r="26" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="7"/>
       <c r="B26" s="59">
         <v>10</v>
       </c>
       <c r="C26" s="55"/>
-      <c r="D26" s="85"/>
-      <c r="E26" s="86"/>
+      <c r="D26" s="81"/>
+      <c r="E26" s="82"/>
       <c r="F26" s="63"/>
       <c r="G26" s="64"/>
       <c r="H26" s="64"/>
@@ -2696,22 +2697,22 @@
       <c r="Q26" s="75"/>
       <c r="R26" s="48"/>
       <c r="S26" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T26" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U26" s="77"/>
-      <c r="V26" s="77"/>
-    </row>
-    <row r="27" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U26" s="117"/>
+      <c r="V26" s="117"/>
+    </row>
+    <row r="27" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="7"/>
       <c r="B27" s="58">
         <v>11</v>
       </c>
       <c r="C27" s="56"/>
-      <c r="D27" s="83"/>
-      <c r="E27" s="84"/>
+      <c r="D27" s="79"/>
+      <c r="E27" s="80"/>
       <c r="F27" s="61"/>
       <c r="G27" s="62"/>
       <c r="H27" s="62"/>
@@ -2729,22 +2730,22 @@
       <c r="Q27" s="76"/>
       <c r="R27" s="40"/>
       <c r="S27" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T27" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U27" s="78"/>
-      <c r="V27" s="78"/>
-    </row>
-    <row r="28" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U27" s="116"/>
+      <c r="V27" s="116"/>
+    </row>
+    <row r="28" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A28" s="7"/>
       <c r="B28" s="59">
         <v>12</v>
       </c>
       <c r="C28" s="55"/>
-      <c r="D28" s="85"/>
-      <c r="E28" s="86"/>
+      <c r="D28" s="81"/>
+      <c r="E28" s="82"/>
       <c r="F28" s="63"/>
       <c r="G28" s="64"/>
       <c r="H28" s="64"/>
@@ -2762,22 +2763,22 @@
       <c r="Q28" s="75"/>
       <c r="R28" s="48"/>
       <c r="S28" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T28" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U28" s="77"/>
-      <c r="V28" s="77"/>
-    </row>
-    <row r="29" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U28" s="117"/>
+      <c r="V28" s="117"/>
+    </row>
+    <row r="29" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A29" s="7"/>
       <c r="B29" s="58">
         <v>13</v>
       </c>
       <c r="C29" s="56"/>
-      <c r="D29" s="83"/>
-      <c r="E29" s="84"/>
+      <c r="D29" s="79"/>
+      <c r="E29" s="80"/>
       <c r="F29" s="61"/>
       <c r="G29" s="62"/>
       <c r="H29" s="62"/>
@@ -2795,22 +2796,22 @@
       <c r="Q29" s="76"/>
       <c r="R29" s="40"/>
       <c r="S29" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T29" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U29" s="78"/>
-      <c r="V29" s="78"/>
-    </row>
-    <row r="30" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U29" s="116"/>
+      <c r="V29" s="116"/>
+    </row>
+    <row r="30" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A30" s="7"/>
       <c r="B30" s="59">
         <v>14</v>
       </c>
       <c r="C30" s="55"/>
-      <c r="D30" s="85"/>
-      <c r="E30" s="86"/>
+      <c r="D30" s="81"/>
+      <c r="E30" s="82"/>
       <c r="F30" s="63"/>
       <c r="G30" s="64"/>
       <c r="H30" s="64"/>
@@ -2828,22 +2829,22 @@
       <c r="Q30" s="75"/>
       <c r="R30" s="48"/>
       <c r="S30" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T30" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U30" s="77"/>
-      <c r="V30" s="77"/>
-    </row>
-    <row r="31" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U30" s="117"/>
+      <c r="V30" s="117"/>
+    </row>
+    <row r="31" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A31" s="7"/>
       <c r="B31" s="58">
         <v>15</v>
       </c>
       <c r="C31" s="56"/>
-      <c r="D31" s="83"/>
-      <c r="E31" s="84"/>
+      <c r="D31" s="79"/>
+      <c r="E31" s="80"/>
       <c r="F31" s="61"/>
       <c r="G31" s="62"/>
       <c r="H31" s="62"/>
@@ -2861,21 +2862,21 @@
       <c r="Q31" s="76"/>
       <c r="R31" s="40"/>
       <c r="S31" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T31" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U31" s="78"/>
-      <c r="V31" s="78"/>
-    </row>
-    <row r="32" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U31" s="116"/>
+      <c r="V31" s="116"/>
+    </row>
+    <row r="32" spans="1:22" ht="34.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B32" s="59">
         <v>16</v>
       </c>
       <c r="C32" s="55"/>
-      <c r="D32" s="85"/>
-      <c r="E32" s="86"/>
+      <c r="D32" s="81"/>
+      <c r="E32" s="82"/>
       <c r="F32" s="63"/>
       <c r="G32" s="64"/>
       <c r="H32" s="64"/>
@@ -2893,21 +2894,21 @@
       <c r="Q32" s="75"/>
       <c r="R32" s="48"/>
       <c r="S32" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T32" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U32" s="77"/>
-      <c r="V32" s="77"/>
-    </row>
-    <row r="33" spans="2:22" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U32" s="117"/>
+      <c r="V32" s="117"/>
+    </row>
+    <row r="33" spans="2:22" ht="39.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B33" s="58">
         <v>17</v>
       </c>
       <c r="C33" s="56"/>
-      <c r="D33" s="83"/>
-      <c r="E33" s="84"/>
+      <c r="D33" s="79"/>
+      <c r="E33" s="80"/>
       <c r="F33" s="61"/>
       <c r="G33" s="62"/>
       <c r="H33" s="62"/>
@@ -2925,21 +2926,21 @@
       <c r="Q33" s="76"/>
       <c r="R33" s="40"/>
       <c r="S33" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T33" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U33" s="78"/>
-      <c r="V33" s="78"/>
-    </row>
-    <row r="34" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U33" s="116"/>
+      <c r="V33" s="116"/>
+    </row>
+    <row r="34" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B34" s="59">
         <v>18</v>
       </c>
       <c r="C34" s="55"/>
-      <c r="D34" s="85"/>
-      <c r="E34" s="86"/>
+      <c r="D34" s="81"/>
+      <c r="E34" s="82"/>
       <c r="F34" s="63"/>
       <c r="G34" s="64"/>
       <c r="H34" s="64"/>
@@ -2957,21 +2958,21 @@
       <c r="Q34" s="75"/>
       <c r="R34" s="48"/>
       <c r="S34" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T34" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U34" s="77"/>
-      <c r="V34" s="77"/>
-    </row>
-    <row r="35" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U34" s="117"/>
+      <c r="V34" s="117"/>
+    </row>
+    <row r="35" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="58">
         <v>19</v>
       </c>
       <c r="C35" s="56"/>
-      <c r="D35" s="83"/>
-      <c r="E35" s="84"/>
+      <c r="D35" s="79"/>
+      <c r="E35" s="80"/>
       <c r="F35" s="61"/>
       <c r="G35" s="62"/>
       <c r="H35" s="62"/>
@@ -2989,21 +2990,21 @@
       <c r="Q35" s="76"/>
       <c r="R35" s="40"/>
       <c r="S35" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T35" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U35" s="78"/>
-      <c r="V35" s="78"/>
-    </row>
-    <row r="36" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U35" s="116"/>
+      <c r="V35" s="116"/>
+    </row>
+    <row r="36" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B36" s="59">
         <v>20</v>
       </c>
       <c r="C36" s="55"/>
-      <c r="D36" s="85"/>
-      <c r="E36" s="86"/>
+      <c r="D36" s="81"/>
+      <c r="E36" s="82"/>
       <c r="F36" s="63"/>
       <c r="G36" s="64"/>
       <c r="H36" s="64"/>
@@ -3021,21 +3022,21 @@
       <c r="Q36" s="75"/>
       <c r="R36" s="48"/>
       <c r="S36" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T36" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U36" s="77"/>
-      <c r="V36" s="77"/>
-    </row>
-    <row r="37" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U36" s="117"/>
+      <c r="V36" s="117"/>
+    </row>
+    <row r="37" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B37" s="58">
         <v>21</v>
       </c>
       <c r="C37" s="56"/>
-      <c r="D37" s="83"/>
-      <c r="E37" s="84"/>
+      <c r="D37" s="79"/>
+      <c r="E37" s="80"/>
       <c r="F37" s="61"/>
       <c r="G37" s="62"/>
       <c r="H37" s="62"/>
@@ -3053,21 +3054,21 @@
       <c r="Q37" s="76"/>
       <c r="R37" s="40"/>
       <c r="S37" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T37" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U37" s="78"/>
-      <c r="V37" s="78"/>
-    </row>
-    <row r="38" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U37" s="116"/>
+      <c r="V37" s="116"/>
+    </row>
+    <row r="38" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B38" s="59">
         <v>22</v>
       </c>
       <c r="C38" s="55"/>
-      <c r="D38" s="85"/>
-      <c r="E38" s="86"/>
+      <c r="D38" s="81"/>
+      <c r="E38" s="82"/>
       <c r="F38" s="63"/>
       <c r="G38" s="64"/>
       <c r="H38" s="64"/>
@@ -3085,21 +3086,21 @@
       <c r="Q38" s="75"/>
       <c r="R38" s="48"/>
       <c r="S38" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T38" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U38" s="77"/>
-      <c r="V38" s="77"/>
-    </row>
-    <row r="39" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U38" s="117"/>
+      <c r="V38" s="117"/>
+    </row>
+    <row r="39" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B39" s="58">
         <v>23</v>
       </c>
       <c r="C39" s="56"/>
-      <c r="D39" s="83"/>
-      <c r="E39" s="84"/>
+      <c r="D39" s="79"/>
+      <c r="E39" s="80"/>
       <c r="F39" s="61"/>
       <c r="G39" s="62"/>
       <c r="H39" s="62"/>
@@ -3117,21 +3118,21 @@
       <c r="Q39" s="76"/>
       <c r="R39" s="40"/>
       <c r="S39" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T39" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U39" s="78"/>
-      <c r="V39" s="78"/>
-    </row>
-    <row r="40" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U39" s="116"/>
+      <c r="V39" s="116"/>
+    </row>
+    <row r="40" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B40" s="59">
         <v>24</v>
       </c>
       <c r="C40" s="55"/>
-      <c r="D40" s="85"/>
-      <c r="E40" s="86"/>
+      <c r="D40" s="81"/>
+      <c r="E40" s="82"/>
       <c r="F40" s="63"/>
       <c r="G40" s="64"/>
       <c r="H40" s="64"/>
@@ -3149,21 +3150,21 @@
       <c r="Q40" s="75"/>
       <c r="R40" s="48"/>
       <c r="S40" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T40" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U40" s="77"/>
-      <c r="V40" s="77"/>
-    </row>
-    <row r="41" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U40" s="117"/>
+      <c r="V40" s="117"/>
+    </row>
+    <row r="41" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B41" s="58">
         <v>25</v>
       </c>
       <c r="C41" s="56"/>
-      <c r="D41" s="83"/>
-      <c r="E41" s="84"/>
+      <c r="D41" s="79"/>
+      <c r="E41" s="80"/>
       <c r="F41" s="61"/>
       <c r="G41" s="62"/>
       <c r="H41" s="62"/>
@@ -3181,21 +3182,21 @@
       <c r="Q41" s="76"/>
       <c r="R41" s="40"/>
       <c r="S41" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T41" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U41" s="78"/>
-      <c r="V41" s="78"/>
-    </row>
-    <row r="42" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U41" s="116"/>
+      <c r="V41" s="116"/>
+    </row>
+    <row r="42" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B42" s="59">
         <v>26</v>
       </c>
       <c r="C42" s="55"/>
-      <c r="D42" s="85"/>
-      <c r="E42" s="86"/>
+      <c r="D42" s="81"/>
+      <c r="E42" s="82"/>
       <c r="F42" s="63"/>
       <c r="G42" s="64"/>
       <c r="H42" s="64"/>
@@ -3213,21 +3214,21 @@
       <c r="Q42" s="75"/>
       <c r="R42" s="48"/>
       <c r="S42" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T42" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U42" s="77"/>
-      <c r="V42" s="77"/>
-    </row>
-    <row r="43" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U42" s="117"/>
+      <c r="V42" s="117"/>
+    </row>
+    <row r="43" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B43" s="58">
         <v>27</v>
       </c>
       <c r="C43" s="56"/>
-      <c r="D43" s="83"/>
-      <c r="E43" s="84"/>
+      <c r="D43" s="79"/>
+      <c r="E43" s="80"/>
       <c r="F43" s="61"/>
       <c r="G43" s="62"/>
       <c r="H43" s="62"/>
@@ -3245,21 +3246,21 @@
       <c r="Q43" s="76"/>
       <c r="R43" s="40"/>
       <c r="S43" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T43" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U43" s="78"/>
-      <c r="V43" s="78"/>
-    </row>
-    <row r="44" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U43" s="116"/>
+      <c r="V43" s="116"/>
+    </row>
+    <row r="44" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B44" s="59">
         <v>28</v>
       </c>
       <c r="C44" s="55"/>
-      <c r="D44" s="85"/>
-      <c r="E44" s="86"/>
+      <c r="D44" s="81"/>
+      <c r="E44" s="82"/>
       <c r="F44" s="63"/>
       <c r="G44" s="64"/>
       <c r="H44" s="64"/>
@@ -3277,21 +3278,21 @@
       <c r="Q44" s="75"/>
       <c r="R44" s="48"/>
       <c r="S44" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T44" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U44" s="77"/>
-      <c r="V44" s="77"/>
-    </row>
-    <row r="45" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U44" s="117"/>
+      <c r="V44" s="117"/>
+    </row>
+    <row r="45" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B45" s="58">
         <v>29</v>
       </c>
       <c r="C45" s="56"/>
-      <c r="D45" s="83"/>
-      <c r="E45" s="84"/>
+      <c r="D45" s="79"/>
+      <c r="E45" s="80"/>
       <c r="F45" s="61"/>
       <c r="G45" s="62"/>
       <c r="H45" s="62"/>
@@ -3309,21 +3310,21 @@
       <c r="Q45" s="76"/>
       <c r="R45" s="40"/>
       <c r="S45" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T45" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U45" s="78"/>
-      <c r="V45" s="78"/>
-    </row>
-    <row r="46" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U45" s="116"/>
+      <c r="V45" s="116"/>
+    </row>
+    <row r="46" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B46" s="59">
         <v>30</v>
       </c>
       <c r="C46" s="55"/>
-      <c r="D46" s="85"/>
-      <c r="E46" s="86"/>
+      <c r="D46" s="81"/>
+      <c r="E46" s="82"/>
       <c r="F46" s="63"/>
       <c r="G46" s="64"/>
       <c r="H46" s="64"/>
@@ -3341,21 +3342,21 @@
       <c r="Q46" s="75"/>
       <c r="R46" s="48"/>
       <c r="S46" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T46" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U46" s="77"/>
-      <c r="V46" s="77"/>
-    </row>
-    <row r="47" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U46" s="117"/>
+      <c r="V46" s="117"/>
+    </row>
+    <row r="47" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B47" s="58">
         <v>31</v>
       </c>
       <c r="C47" s="56"/>
-      <c r="D47" s="83"/>
-      <c r="E47" s="84"/>
+      <c r="D47" s="79"/>
+      <c r="E47" s="80"/>
       <c r="F47" s="61"/>
       <c r="G47" s="62"/>
       <c r="H47" s="62"/>
@@ -3373,21 +3374,21 @@
       <c r="Q47" s="76"/>
       <c r="R47" s="40"/>
       <c r="S47" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T47" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U47" s="78"/>
-      <c r="V47" s="78"/>
-    </row>
-    <row r="48" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U47" s="116"/>
+      <c r="V47" s="116"/>
+    </row>
+    <row r="48" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B48" s="59">
         <v>32</v>
       </c>
       <c r="C48" s="55"/>
-      <c r="D48" s="85"/>
-      <c r="E48" s="86"/>
+      <c r="D48" s="81"/>
+      <c r="E48" s="82"/>
       <c r="F48" s="63"/>
       <c r="G48" s="64"/>
       <c r="H48" s="64"/>
@@ -3405,21 +3406,21 @@
       <c r="Q48" s="75"/>
       <c r="R48" s="48"/>
       <c r="S48" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T48" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U48" s="77"/>
-      <c r="V48" s="77"/>
-    </row>
-    <row r="49" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U48" s="117"/>
+      <c r="V48" s="117"/>
+    </row>
+    <row r="49" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B49" s="58">
         <v>33</v>
       </c>
       <c r="C49" s="56"/>
-      <c r="D49" s="83"/>
-      <c r="E49" s="84"/>
+      <c r="D49" s="79"/>
+      <c r="E49" s="80"/>
       <c r="F49" s="61"/>
       <c r="G49" s="62"/>
       <c r="H49" s="62"/>
@@ -3437,21 +3438,21 @@
       <c r="Q49" s="76"/>
       <c r="R49" s="40"/>
       <c r="S49" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T49" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U49" s="78"/>
-      <c r="V49" s="78"/>
-    </row>
-    <row r="50" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U49" s="116"/>
+      <c r="V49" s="116"/>
+    </row>
+    <row r="50" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B50" s="59">
         <v>34</v>
       </c>
       <c r="C50" s="55"/>
-      <c r="D50" s="85"/>
-      <c r="E50" s="86"/>
+      <c r="D50" s="81"/>
+      <c r="E50" s="82"/>
       <c r="F50" s="63"/>
       <c r="G50" s="64"/>
       <c r="H50" s="64"/>
@@ -3469,21 +3470,21 @@
       <c r="Q50" s="75"/>
       <c r="R50" s="48"/>
       <c r="S50" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T50" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U50" s="77"/>
-      <c r="V50" s="77"/>
-    </row>
-    <row r="51" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U50" s="117"/>
+      <c r="V50" s="117"/>
+    </row>
+    <row r="51" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B51" s="58">
         <v>35</v>
       </c>
       <c r="C51" s="56"/>
-      <c r="D51" s="83"/>
-      <c r="E51" s="84"/>
+      <c r="D51" s="79"/>
+      <c r="E51" s="80"/>
       <c r="F51" s="61"/>
       <c r="G51" s="62"/>
       <c r="H51" s="62"/>
@@ -3501,21 +3502,21 @@
       <c r="Q51" s="76"/>
       <c r="R51" s="40"/>
       <c r="S51" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T51" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U51" s="78"/>
-      <c r="V51" s="78"/>
-    </row>
-    <row r="52" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U51" s="116"/>
+      <c r="V51" s="116"/>
+    </row>
+    <row r="52" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B52" s="59">
         <v>36</v>
       </c>
       <c r="C52" s="55"/>
-      <c r="D52" s="85"/>
-      <c r="E52" s="86"/>
+      <c r="D52" s="81"/>
+      <c r="E52" s="82"/>
       <c r="F52" s="63"/>
       <c r="G52" s="64"/>
       <c r="H52" s="64"/>
@@ -3533,21 +3534,21 @@
       <c r="Q52" s="75"/>
       <c r="R52" s="48"/>
       <c r="S52" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T52" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U52" s="77"/>
-      <c r="V52" s="77"/>
-    </row>
-    <row r="53" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U52" s="117"/>
+      <c r="V52" s="117"/>
+    </row>
+    <row r="53" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B53" s="58">
         <v>37</v>
       </c>
       <c r="C53" s="56"/>
-      <c r="D53" s="83"/>
-      <c r="E53" s="84"/>
+      <c r="D53" s="79"/>
+      <c r="E53" s="80"/>
       <c r="F53" s="61"/>
       <c r="G53" s="62"/>
       <c r="H53" s="62"/>
@@ -3565,21 +3566,21 @@
       <c r="Q53" s="76"/>
       <c r="R53" s="40"/>
       <c r="S53" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T53" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U53" s="78"/>
-      <c r="V53" s="78"/>
-    </row>
-    <row r="54" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U53" s="116"/>
+      <c r="V53" s="116"/>
+    </row>
+    <row r="54" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B54" s="59">
         <v>38</v>
       </c>
       <c r="C54" s="55"/>
-      <c r="D54" s="85"/>
-      <c r="E54" s="86"/>
+      <c r="D54" s="81"/>
+      <c r="E54" s="82"/>
       <c r="F54" s="63"/>
       <c r="G54" s="64"/>
       <c r="H54" s="64"/>
@@ -3597,21 +3598,21 @@
       <c r="Q54" s="75"/>
       <c r="R54" s="48"/>
       <c r="S54" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T54" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U54" s="77"/>
-      <c r="V54" s="77"/>
-    </row>
-    <row r="55" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U54" s="117"/>
+      <c r="V54" s="117"/>
+    </row>
+    <row r="55" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B55" s="58">
         <v>39</v>
       </c>
       <c r="C55" s="56"/>
-      <c r="D55" s="83"/>
-      <c r="E55" s="84"/>
+      <c r="D55" s="79"/>
+      <c r="E55" s="80"/>
       <c r="F55" s="61"/>
       <c r="G55" s="62"/>
       <c r="H55" s="62"/>
@@ -3629,21 +3630,21 @@
       <c r="Q55" s="76"/>
       <c r="R55" s="40"/>
       <c r="S55" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T55" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U55" s="78"/>
-      <c r="V55" s="78"/>
-    </row>
-    <row r="56" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U55" s="116"/>
+      <c r="V55" s="116"/>
+    </row>
+    <row r="56" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B56" s="59">
         <v>40</v>
       </c>
       <c r="C56" s="55"/>
-      <c r="D56" s="85"/>
-      <c r="E56" s="86"/>
+      <c r="D56" s="81"/>
+      <c r="E56" s="82"/>
       <c r="F56" s="63"/>
       <c r="G56" s="64"/>
       <c r="H56" s="64"/>
@@ -3661,21 +3662,21 @@
       <c r="Q56" s="75"/>
       <c r="R56" s="48"/>
       <c r="S56" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T56" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U56" s="77"/>
-      <c r="V56" s="77"/>
-    </row>
-    <row r="57" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U56" s="117"/>
+      <c r="V56" s="117"/>
+    </row>
+    <row r="57" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B57" s="58">
         <v>41</v>
       </c>
       <c r="C57" s="56"/>
-      <c r="D57" s="83"/>
-      <c r="E57" s="84"/>
+      <c r="D57" s="79"/>
+      <c r="E57" s="80"/>
       <c r="F57" s="61"/>
       <c r="G57" s="62"/>
       <c r="H57" s="62"/>
@@ -3693,21 +3694,21 @@
       <c r="Q57" s="76"/>
       <c r="R57" s="40"/>
       <c r="S57" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T57" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U57" s="78"/>
-      <c r="V57" s="78"/>
-    </row>
-    <row r="58" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U57" s="116"/>
+      <c r="V57" s="116"/>
+    </row>
+    <row r="58" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B58" s="59">
         <v>42</v>
       </c>
       <c r="C58" s="55"/>
-      <c r="D58" s="85"/>
-      <c r="E58" s="86"/>
+      <c r="D58" s="81"/>
+      <c r="E58" s="82"/>
       <c r="F58" s="63"/>
       <c r="G58" s="64"/>
       <c r="H58" s="64"/>
@@ -3725,21 +3726,21 @@
       <c r="Q58" s="75"/>
       <c r="R58" s="48"/>
       <c r="S58" s="53" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T58" s="53" t="s">
-        <v>39</v>
-      </c>
-      <c r="U58" s="77"/>
-      <c r="V58" s="77"/>
-    </row>
-    <row r="59" spans="2:22" ht="37.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+      <c r="U58" s="117"/>
+      <c r="V58" s="117"/>
+    </row>
+    <row r="59" spans="2:22" ht="38" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B59" s="58">
         <v>43</v>
       </c>
       <c r="C59" s="56"/>
-      <c r="D59" s="83"/>
-      <c r="E59" s="84"/>
+      <c r="D59" s="79"/>
+      <c r="E59" s="80"/>
       <c r="F59" s="61"/>
       <c r="G59" s="62"/>
       <c r="H59" s="62"/>
@@ -3757,55 +3758,64 @@
       <c r="Q59" s="76"/>
       <c r="R59" s="40"/>
       <c r="S59" s="45" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="T59" s="45" t="s">
-        <v>39</v>
-      </c>
-      <c r="U59" s="78"/>
-      <c r="V59" s="78"/>
+        <v>38</v>
+      </c>
+      <c r="U59" s="116"/>
+      <c r="V59" s="116"/>
     </row>
   </sheetData>
   <protectedRanges>
     <protectedRange sqref="C16:U59" name="範囲1"/>
   </protectedRanges>
   <mergeCells count="105">
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="D58:E58"/>
-    <mergeCell ref="D59:E59"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="D55:E55"/>
-    <mergeCell ref="D56:E56"/>
-    <mergeCell ref="D57:E57"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="D42:E42"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="T1:U2"/>
-    <mergeCell ref="B12:B14"/>
-    <mergeCell ref="C12:C14"/>
-    <mergeCell ref="D12:E14"/>
-    <mergeCell ref="F12:L12"/>
-    <mergeCell ref="M12:M14"/>
-    <mergeCell ref="N12:P12"/>
-    <mergeCell ref="R12:R14"/>
-    <mergeCell ref="S12:S14"/>
-    <mergeCell ref="T12:T14"/>
-    <mergeCell ref="N13:P13"/>
-    <mergeCell ref="U12:V14"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="Q12:Q14"/>
+    <mergeCell ref="U56:V56"/>
+    <mergeCell ref="U57:V57"/>
+    <mergeCell ref="U58:V58"/>
+    <mergeCell ref="U59:V59"/>
+    <mergeCell ref="U16:V16"/>
+    <mergeCell ref="U51:V51"/>
+    <mergeCell ref="U52:V52"/>
+    <mergeCell ref="U53:V53"/>
+    <mergeCell ref="U54:V54"/>
+    <mergeCell ref="U55:V55"/>
+    <mergeCell ref="U46:V46"/>
+    <mergeCell ref="U47:V47"/>
+    <mergeCell ref="U48:V48"/>
+    <mergeCell ref="U49:V49"/>
+    <mergeCell ref="U50:V50"/>
+    <mergeCell ref="U41:V41"/>
+    <mergeCell ref="U42:V42"/>
+    <mergeCell ref="U43:V43"/>
+    <mergeCell ref="U44:V44"/>
+    <mergeCell ref="U45:V45"/>
+    <mergeCell ref="U36:V36"/>
+    <mergeCell ref="U37:V37"/>
+    <mergeCell ref="U38:V38"/>
+    <mergeCell ref="U39:V39"/>
+    <mergeCell ref="U40:V40"/>
+    <mergeCell ref="U31:V31"/>
+    <mergeCell ref="U32:V32"/>
+    <mergeCell ref="U33:V33"/>
+    <mergeCell ref="U34:V34"/>
+    <mergeCell ref="U35:V35"/>
+    <mergeCell ref="U26:V26"/>
+    <mergeCell ref="U27:V27"/>
+    <mergeCell ref="U28:V28"/>
+    <mergeCell ref="U29:V29"/>
+    <mergeCell ref="U30:V30"/>
+    <mergeCell ref="U21:V21"/>
+    <mergeCell ref="U22:V22"/>
+    <mergeCell ref="U23:V23"/>
+    <mergeCell ref="U24:V24"/>
+    <mergeCell ref="U25:V25"/>
+    <mergeCell ref="U15:V15"/>
+    <mergeCell ref="U17:V17"/>
+    <mergeCell ref="U18:V18"/>
+    <mergeCell ref="U19:V19"/>
+    <mergeCell ref="U20:V20"/>
     <mergeCell ref="D35:E35"/>
     <mergeCell ref="D36:E36"/>
     <mergeCell ref="D37:E37"/>
@@ -3830,51 +3840,42 @@
     <mergeCell ref="D25:E25"/>
     <mergeCell ref="D26:E26"/>
     <mergeCell ref="D27:E27"/>
-    <mergeCell ref="U21:V21"/>
-    <mergeCell ref="U22:V22"/>
-    <mergeCell ref="U23:V23"/>
-    <mergeCell ref="U24:V24"/>
-    <mergeCell ref="U25:V25"/>
-    <mergeCell ref="U15:V15"/>
-    <mergeCell ref="U17:V17"/>
-    <mergeCell ref="U18:V18"/>
-    <mergeCell ref="U19:V19"/>
-    <mergeCell ref="U20:V20"/>
-    <mergeCell ref="U40:V40"/>
-    <mergeCell ref="U31:V31"/>
-    <mergeCell ref="U32:V32"/>
-    <mergeCell ref="U33:V33"/>
-    <mergeCell ref="U34:V34"/>
-    <mergeCell ref="U35:V35"/>
-    <mergeCell ref="U26:V26"/>
-    <mergeCell ref="U27:V27"/>
-    <mergeCell ref="U28:V28"/>
-    <mergeCell ref="U29:V29"/>
-    <mergeCell ref="U30:V30"/>
-    <mergeCell ref="U56:V56"/>
-    <mergeCell ref="U57:V57"/>
-    <mergeCell ref="U58:V58"/>
-    <mergeCell ref="U59:V59"/>
-    <mergeCell ref="U16:V16"/>
-    <mergeCell ref="U51:V51"/>
-    <mergeCell ref="U52:V52"/>
-    <mergeCell ref="U53:V53"/>
-    <mergeCell ref="U54:V54"/>
-    <mergeCell ref="U55:V55"/>
-    <mergeCell ref="U46:V46"/>
-    <mergeCell ref="U47:V47"/>
-    <mergeCell ref="U48:V48"/>
-    <mergeCell ref="U49:V49"/>
-    <mergeCell ref="U50:V50"/>
-    <mergeCell ref="U41:V41"/>
-    <mergeCell ref="U42:V42"/>
-    <mergeCell ref="U43:V43"/>
-    <mergeCell ref="U44:V44"/>
-    <mergeCell ref="U45:V45"/>
-    <mergeCell ref="U36:V36"/>
-    <mergeCell ref="U37:V37"/>
-    <mergeCell ref="U38:V38"/>
-    <mergeCell ref="U39:V39"/>
+    <mergeCell ref="T1:U2"/>
+    <mergeCell ref="B12:B14"/>
+    <mergeCell ref="C12:C14"/>
+    <mergeCell ref="D12:E14"/>
+    <mergeCell ref="F12:L12"/>
+    <mergeCell ref="M12:M14"/>
+    <mergeCell ref="N12:P12"/>
+    <mergeCell ref="R12:R14"/>
+    <mergeCell ref="S12:S14"/>
+    <mergeCell ref="T12:T14"/>
+    <mergeCell ref="N13:P13"/>
+    <mergeCell ref="U12:V14"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="Q12:Q14"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="D42:E42"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="D58:E58"/>
+    <mergeCell ref="D59:E59"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="D54:E54"/>
+    <mergeCell ref="D55:E55"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="D57:E57"/>
   </mergeCells>
   <phoneticPr fontId="2"/>
   <dataValidations count="1">
@@ -3892,15 +3893,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="ドキュメント" ma:contentTypeID="0x01010071CCB8D28BC6C44EA501C00017828CA7" ma:contentTypeVersion="10" ma:contentTypeDescription="新しいドキュメントを作成します。" ma:contentTypeScope="" ma:versionID="630046f5d86abb6f6a211bf3773a49b3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="e07dd695-b70d-4177-bfc3-4750b24c049d" xmlns:ns3="afd4e677-d9f8-4eb2-a5b6-468f89fa9c12" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bea37b67cd06610812e20ccc94c5f34d" ns2:_="" ns3:_="">
     <xsd:import namespace="e07dd695-b70d-4177-bfc3-4750b24c049d"/>
@@ -4089,6 +4081,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -4101,15 +4102,30 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2C0D765-70AD-4C94-A4D6-A2494E34688F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="e07dd695-b70d-4177-bfc3-4750b24c049d"/>
+    <ds:schemaRef ds:uri="afd4e677-d9f8-4eb2-a5b6-468f89fa9c12"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{868AD63B-67FA-426B-B925-0B97DF7CF326}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E2C0D765-70AD-4C94-A4D6-A2494E34688F}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -4124,6 +4140,8 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="543e2540-031c-428b-a0d9-09b0ecfc5dce"/>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="e07dd695-b70d-4177-bfc3-4750b24c049d"/>
+    <ds:schemaRef ds:uri="afd4e677-d9f8-4eb2-a5b6-468f89fa9c12"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>